<commit_message>
Added rest of the login tests
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/DDT.xlsx
+++ b/src/test/java/TestData/DDT.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Username</t>
   </si>
@@ -86,6 +86,12 @@
   </si>
   <si>
     <t>standard_user</t>
+  </si>
+  <si>
+    <t>invalid_password</t>
+  </si>
+  <si>
+    <t>invalid_username</t>
   </si>
 </sst>
 </file>
@@ -427,11 +433,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -472,6 +478,9 @@
       <c r="A3" t="s">
         <v>5</v>
       </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -521,6 +530,11 @@
       </c>
       <c r="D7" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added E2E test that user can checkout with item
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/DDT.xlsx
+++ b/src/test/java/TestData/DDT.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Username</t>
   </si>
@@ -92,6 +92,12 @@
   </si>
   <si>
     <t>invalid_username</t>
+  </si>
+  <si>
+    <t>Marija</t>
+  </si>
+  <si>
+    <t>Korac</t>
   </si>
 </sst>
 </file>
@@ -434,13 +440,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,7 +463,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -474,7 +480,7 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -488,7 +494,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -499,7 +505,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -510,7 +516,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -521,7 +527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -532,9 +538,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>